<commit_message>
Added table 23.01.01 as suggested
</commit_message>
<xml_diff>
--- a/master_list_partial.xlsx
+++ b/master_list_partial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Desktop\SFCR_using_Mistral_2025-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6120E6-9CC9-450A-8F1F-28CB411A5A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB92867-7D47-4C9B-B749-AF07F143B6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
+    <workbookView xWindow="36225" yWindow="735" windowWidth="19200" windowHeight="10185" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
   </bookViews>
   <sheets>
     <sheet name="ITALY_2025" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>company</t>
   </si>
@@ -132,6 +132,42 @@
   </si>
   <si>
     <t>sfcr-2025_ca-vita.pdf</t>
+  </si>
+  <si>
+    <t>AXA_VITA_23_01</t>
+  </si>
+  <si>
+    <t>S_23_01_01</t>
+  </si>
+  <si>
+    <t>GEN_ITA_23_01</t>
+  </si>
+  <si>
+    <t>B_ITA</t>
+  </si>
+  <si>
+    <t>HDI_23_01</t>
+  </si>
+  <si>
+    <t>ZURICH_LIFE_23_01_01</t>
+  </si>
+  <si>
+    <t>ZURICH_LIFE_23_01_02</t>
+  </si>
+  <si>
+    <t>S_23_01_01_1</t>
+  </si>
+  <si>
+    <t>S_23_01_01_2</t>
+  </si>
+  <si>
+    <t>CREDAG_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>CREDAG_VITA_23_01_02</t>
+  </si>
+  <si>
+    <t>table_category</t>
   </si>
 </sst>
 </file>
@@ -511,16 +547,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43813C6-155E-442B-992A-28BDB54378D4}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="31.1796875" customWidth="1"/>
     <col min="3" max="3" width="16.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="78.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -539,8 +576,11 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -559,8 +599,11 @@
       <c r="F2" s="2">
         <v>98</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -579,8 +622,11 @@
       <c r="F3" s="2">
         <v>142</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -599,8 +645,11 @@
       <c r="F4" s="2">
         <v>143</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -619,8 +668,11 @@
       <c r="F5" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -639,8 +691,11 @@
       <c r="F6" s="2">
         <v>101</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -659,8 +714,11 @@
       <c r="F7" s="2">
         <v>58</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -679,8 +737,11 @@
       <c r="F8" s="2">
         <v>59</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G8" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
@@ -699,8 +760,11 @@
       <c r="F9" s="2">
         <v>64</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -718,6 +782,170 @@
       </c>
       <c r="F10" s="2">
         <v>65</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="2">
+        <v>103</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="2">
+        <v>162</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="2">
+        <v>108</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="2">
+        <v>67</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" s="2">
+        <v>68</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="2">
+        <v>70</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="2">
+        <v>71</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code with validation of S.02.01.02
</commit_message>
<xml_diff>
--- a/master_list_partial.xlsx
+++ b/master_list_partial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Desktop\SFCR_using_Mistral_2025-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB92867-7D47-4C9B-B749-AF07F143B6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C276CC-E0C0-4932-B367-97096152B79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36225" yWindow="735" windowWidth="19200" windowHeight="10185" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
+    <workbookView xWindow="3600" yWindow="3600" windowWidth="19200" windowHeight="11170" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
   </bookViews>
   <sheets>
     <sheet name="ITALY_2025" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="60">
   <si>
     <t>company</t>
   </si>
@@ -168,6 +168,57 @@
   </si>
   <si>
     <t>table_category</t>
+  </si>
+  <si>
+    <t>CREDEM_VITA_02_1</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>CREDEM_VITA</t>
+  </si>
+  <si>
+    <t>CREDEM_VITA_02_2</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>CREDEM_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>CREDEM_VITA_23_01_02</t>
+  </si>
+  <si>
+    <t>SFCR al 31 Dicembre 2025.pdf</t>
+  </si>
+  <si>
+    <t>CARDIF_02_01</t>
+  </si>
+  <si>
+    <t>CARDIF</t>
+  </si>
+  <si>
+    <t>CARDIF_23_01_01</t>
+  </si>
+  <si>
+    <t>HELVETIA_VITA_01</t>
+  </si>
+  <si>
+    <t>HELVETIA_VITA</t>
+  </si>
+  <si>
+    <t>HELVETIA_VITA_02</t>
+  </si>
+  <si>
+    <t>Relazione-sulla-Solvibilita-e-Condizione-Finanziaria-2025.pdf</t>
+  </si>
+  <si>
+    <t>SFCR-Annex_Helvetia Vita_2025.pdf</t>
+  </si>
+  <si>
+    <t>HELVETIA_VITA_23_01_01</t>
   </si>
 </sst>
 </file>
@@ -209,10 +260,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43813C6-155E-442B-992A-28BDB54378D4}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="31.1796875" customWidth="1"/>
@@ -788,138 +840,138 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="3">
+        <v>172</v>
+      </c>
+      <c r="G11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="3">
+        <v>173</v>
+      </c>
+      <c r="G12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11" s="2">
-        <v>103</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="2">
-        <v>162</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" s="2">
-        <v>108</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>32</v>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="3">
+        <v>113</v>
+      </c>
+      <c r="G13" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F14" s="2">
-        <v>67</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>32</v>
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="3">
+        <v>2</v>
+      </c>
+      <c r="G14" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="2">
-        <v>68</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>32</v>
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="3">
+        <v>3</v>
+      </c>
+      <c r="G15" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F16" s="2">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>32</v>
@@ -927,24 +979,231 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="2">
+        <v>162</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="2">
+        <v>108</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="2">
+        <v>67</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="2">
+        <v>68</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="2">
+        <v>70</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F22" s="2">
         <v>71</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F23" s="3">
+        <v>178</v>
+      </c>
+      <c r="G23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="3">
+        <v>179</v>
+      </c>
+      <c r="G24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" s="3">
+        <v>121</v>
+      </c>
+      <c r="G25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="3">
+        <v>8</v>
+      </c>
+      <c r="G26" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
With BMP Vita and UniCredit Life
</commit_message>
<xml_diff>
--- a/master_list_partial.xlsx
+++ b/master_list_partial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Desktop\SFCR_using_Mistral_2025-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C276CC-E0C0-4932-B367-97096152B79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{636DAAFE-8127-43FA-AB48-19664D38947D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="3600" windowWidth="19200" windowHeight="11170" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
   </bookViews>
   <sheets>
     <sheet name="ITALY_2025" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="71">
   <si>
     <t>company</t>
   </si>
@@ -219,6 +219,39 @@
   </si>
   <si>
     <t>HELVETIA_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>BMP_VITA_02_01</t>
+  </si>
+  <si>
+    <t>BMP VITA</t>
+  </si>
+  <si>
+    <t>BMP_VITA_02_02</t>
+  </si>
+  <si>
+    <t>SFCR_BBPMV_202512311.pdf</t>
+  </si>
+  <si>
+    <t>BMP_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>UNICREDIT_VITA_02_01</t>
+  </si>
+  <si>
+    <t>57185-Relazione relativa alla solvibilità e condizione finanziaria SFCR 2025.pdf</t>
+  </si>
+  <si>
+    <t>UNICREDIT VITA</t>
+  </si>
+  <si>
+    <t>UNICREDIT_VITA_02_02</t>
+  </si>
+  <si>
+    <t>UNICREDIT_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>UNICREDIT_VITA_23_01_02</t>
   </si>
 </sst>
 </file>
@@ -599,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43813C6-155E-442B-992A-28BDB54378D4}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="31.1796875" customWidth="1"/>
@@ -955,115 +988,115 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="2">
-        <v>103</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>32</v>
+      <c r="A16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="3">
+        <v>92</v>
+      </c>
+      <c r="G16" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="2">
-        <v>162</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>32</v>
+      <c r="A17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="3">
+        <v>93</v>
+      </c>
+      <c r="G17" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F18" s="2">
-        <v>108</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>32</v>
+      <c r="A18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="3">
+        <v>106</v>
+      </c>
+      <c r="G18" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="2">
+      <c r="A19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
         <v>67</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>32</v>
+      <c r="D19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="3">
+        <v>107</v>
+      </c>
+      <c r="G19" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="F20" s="2">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>32</v>
@@ -1071,22 +1104,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F21" s="2">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>32</v>
@@ -1094,116 +1127,277 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="2">
+        <v>108</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F23" s="2">
+        <v>67</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="2">
+        <v>68</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="2">
+        <v>70</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F26" s="2">
         <v>71</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="G26" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>48</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B27" t="s">
         <v>44</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C27" t="s">
         <v>45</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D27" t="s">
         <v>50</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E27" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F27" s="3">
         <v>178</v>
       </c>
-      <c r="G23" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="G27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>49</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B28" t="s">
         <v>47</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C28" t="s">
         <v>45</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D28" t="s">
         <v>50</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E28" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F28" s="3">
         <v>179</v>
       </c>
-      <c r="G24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="G28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>53</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B29" t="s">
         <v>19</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C29" t="s">
         <v>52</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D29" t="s">
         <v>57</v>
       </c>
-      <c r="E25" t="s">
-        <v>32</v>
-      </c>
-      <c r="F25" s="3">
+      <c r="E29" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="3">
         <v>121</v>
       </c>
-      <c r="G25" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="G29" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>59</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B30" t="s">
         <v>19</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C30" t="s">
         <v>55</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D30" t="s">
         <v>58</v>
       </c>
-      <c r="E26" t="s">
-        <v>32</v>
-      </c>
-      <c r="F26" s="3">
+      <c r="E30" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="3">
         <v>8</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D31" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" t="s">
+        <v>32</v>
+      </c>
+      <c r="F31" s="3">
+        <v>100</v>
+      </c>
+      <c r="G31" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" t="s">
+        <v>66</v>
+      </c>
+      <c r="E32" t="s">
+        <v>38</v>
+      </c>
+      <c r="F32" s="3">
+        <v>111</v>
+      </c>
+      <c r="G32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" t="s">
+        <v>66</v>
+      </c>
+      <c r="E33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F33" s="3">
+        <v>112</v>
+      </c>
+      <c r="G33" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added CNP and Allianz-UniCredit
</commit_message>
<xml_diff>
--- a/master_list_partial.xlsx
+++ b/master_list_partial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Desktop\SFCR_using_Mistral_2025-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{636DAAFE-8127-43FA-AB48-19664D38947D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40086B3-E9D0-468E-8A6B-26ED31F30C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="82">
   <si>
     <t>company</t>
   </si>
@@ -252,6 +252,39 @@
   </si>
   <si>
     <t>UNICREDIT_VITA_23_01_02</t>
+  </si>
+  <si>
+    <t>CNP_VITA</t>
+  </si>
+  <si>
+    <t>CNP_VITA_02_01</t>
+  </si>
+  <si>
+    <t>CNP_VITA_02_02</t>
+  </si>
+  <si>
+    <t>SFCR_CNP_Vita_Assicura_2025.pdf</t>
+  </si>
+  <si>
+    <t>CNP_VITA_23_01_01</t>
+  </si>
+  <si>
+    <t>CNP_VITA_23_01_02</t>
+  </si>
+  <si>
+    <t>ALLIANZ_UNICREDIT</t>
+  </si>
+  <si>
+    <t>ALLIANZ_UNICREDIT_02_01</t>
+  </si>
+  <si>
+    <t>ALLIANZ_UNICREDIT_02_02</t>
+  </si>
+  <si>
+    <t>57265-Relazione_relativa_alla_solvibilita_e_condizione_finanziaria_SFCR_2025_UniCredit_Vita_Assicurazioni.pdf</t>
+  </si>
+  <si>
+    <t>ALLIANZ_UNICREDIT_23_01_01</t>
   </si>
 </sst>
 </file>
@@ -632,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43813C6-155E-442B-992A-28BDB54378D4}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="31.1796875" customWidth="1"/>
@@ -1080,115 +1113,115 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" s="2">
-        <v>103</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>32</v>
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="3">
+        <v>140</v>
+      </c>
+      <c r="G20" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="2">
-        <v>162</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>32</v>
+      <c r="A21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="3">
+        <v>141</v>
+      </c>
+      <c r="G21" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="2">
+      <c r="A22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="3">
+        <v>107</v>
+      </c>
+      <c r="G22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="3">
         <v>108</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="2">
-        <v>67</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>32</v>
+      <c r="G23" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="F24" s="2">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>32</v>
@@ -1196,22 +1229,22 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F25" s="2">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>32</v>
@@ -1219,137 +1252,137 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="2">
+        <v>108</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" s="2">
+        <v>67</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" s="2">
+        <v>68</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="2">
+        <v>70</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F30" s="2">
         <v>71</v>
       </c>
-      <c r="G26" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" t="s">
-        <v>50</v>
-      </c>
-      <c r="E27" t="s">
-        <v>38</v>
-      </c>
-      <c r="F27" s="3">
-        <v>178</v>
-      </c>
-      <c r="G27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" t="s">
-        <v>45</v>
-      </c>
-      <c r="D28" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" t="s">
-        <v>39</v>
-      </c>
-      <c r="F28" s="3">
-        <v>179</v>
-      </c>
-      <c r="G28" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" t="s">
-        <v>52</v>
-      </c>
-      <c r="D29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E29" t="s">
-        <v>32</v>
-      </c>
-      <c r="F29" s="3">
-        <v>121</v>
-      </c>
-      <c r="G29" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" t="s">
-        <v>19</v>
-      </c>
-      <c r="C30" t="s">
-        <v>55</v>
-      </c>
-      <c r="D30" t="s">
-        <v>58</v>
-      </c>
-      <c r="E30" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" s="3">
-        <v>8</v>
-      </c>
-      <c r="G30" t="s">
+      <c r="G30" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="B31" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="D31" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="E31" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F31" s="3">
-        <v>100</v>
+        <v>178</v>
       </c>
       <c r="G31" t="s">
         <v>32</v>
@@ -1357,22 +1390,22 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="D32" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E32" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F32" s="3">
-        <v>111</v>
+        <v>179</v>
       </c>
       <c r="G32" t="s">
         <v>32</v>
@@ -1380,24 +1413,185 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" t="s">
+        <v>32</v>
+      </c>
+      <c r="F33" s="3">
+        <v>121</v>
+      </c>
+      <c r="G33" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" t="s">
+        <v>55</v>
+      </c>
+      <c r="D34" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" t="s">
+        <v>32</v>
+      </c>
+      <c r="F34" s="3">
+        <v>8</v>
+      </c>
+      <c r="G34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" t="s">
+        <v>32</v>
+      </c>
+      <c r="F35" s="3">
+        <v>100</v>
+      </c>
+      <c r="G35" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" t="s">
+        <v>67</v>
+      </c>
+      <c r="D36" t="s">
+        <v>66</v>
+      </c>
+      <c r="E36" t="s">
+        <v>38</v>
+      </c>
+      <c r="F36" s="3">
+        <v>111</v>
+      </c>
+      <c r="G36" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>70</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B37" t="s">
         <v>21</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C37" t="s">
         <v>67</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D37" t="s">
         <v>66</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E37" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F37" s="3">
         <v>112</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G37" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>75</v>
+      </c>
+      <c r="B38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" t="s">
+        <v>38</v>
+      </c>
+      <c r="F38" s="3">
+        <v>145</v>
+      </c>
+      <c r="G38" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" t="s">
+        <v>47</v>
+      </c>
+      <c r="C39" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39" t="s">
+        <v>74</v>
+      </c>
+      <c r="E39" t="s">
+        <v>39</v>
+      </c>
+      <c r="F39" s="3">
+        <v>146</v>
+      </c>
+      <c r="G39" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>81</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" t="s">
+        <v>77</v>
+      </c>
+      <c r="D40" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" t="s">
+        <v>32</v>
+      </c>
+      <c r="F40" s="3">
+        <v>115</v>
+      </c>
+      <c r="G40" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>